<commit_message>
Resserre encounter vers FRCoreEncounterProfile
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com> 14685a7c001dac29b6f0ea77d4fac3bbd960423b
</commit_message>
<xml_diff>
--- a/nr-doc-core-procedure/ig/StructureDefinition-fr-core-procedure.xlsx
+++ b/nr-doc-core-procedure/ig/StructureDefinition-fr-core-procedure.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-22T12:55:33+00:00</t>
+    <t>2026-07-23T09:09:32+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -814,7 +814,7 @@
     <t>Procedure.encounter</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(Encounter|4.0.1)
+    <t xml:space="preserve">Reference(https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-encounter|2.2.0)
 </t>
   </si>
   <si>

</xml_diff>